<commit_message>
Structure of the program into modules
</commit_message>
<xml_diff>
--- a/responses/zero-shot/auswertung.xlsx
+++ b/responses/zero-shot/auswertung.xlsx
@@ -464,14 +464,16 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>| Direktes Zitat \( T_i \) | Bewertung \( f_i \) |
-|--------------------------|---------------------|
-| "Ausgestaltung:  Cognitive-Load-Theorie" | 1 |
-| "Cognitive Theorie of Multimedia Learning (CTML)" | 1 |
-| "ICAP-Modell" | 1 |
-| "Multimediaprinzip: Lernerfolg größer, wenn Bilder und Texte enthalten sind" | 1 |
-| "man sollte Gelegenheiten für interaktive Aktivitäten Schaffen (Gruppenarbeiten)" | 1 |
-| **Gesamtbewertung**      | 5                   |</t>
+          <t>```markdown
+| Direktes Zitat \( T_i \)                                                                  | Bewertung \( f_i \) |
+|------------------------------------------------------------------------------------------|---------------------|
+| "Ausgestaltung:  Cognitive-Load-Theorie"                                                 | 1                   |
+| "Cognitive Theorie of Multimedia Learning (CTML)"                                        | 1                   |
+| "ICAP-Modell"                                                                            | 1                   |
+| "Multimediale Inhalte müssen beide Informationsverarbeitungskanäle ansprechen"           | 1                   |
+| "Lerninhalte sollten nicht einfach nur präsentiert werden, sondern ... interaktive Aktivitäten schaffen" | 1                   |
+| **Gesamtbewertung**                                                                      | 5                   |
+```</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -486,14 +488,14 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>| Direktes Zitat \( T_i \)                                                                                     | Bewertung \( f_i \) |
-|--------------------------------------------------------------------------------------------------------------|---------------------|
-| "cognitive-load-theorie"                                                                                     | 1                   |
-| "Das ICAP-Modell von Chi &amp; Wylie"                                                                            | 1                   |
-| "Die Cognitive Theory of Multimedia Learning (CTML) von Mayer"                                               | 1                   |
-| "Evidenzbasierte Prinzipien zur Gestaltung von multimedialen Inhalten"                                       | 1                   |
-| "daher würde ich alle Lernaktivitäten miteinander vereinen, um den bestmöglichen Vortrag zu haben"            | 1                   |
-| **Gesamtbewertung**                                                                                          | 5                   |</t>
+          <t>| Direktes Zitat \( T_i \)                                                                                                                                                                                                                                                                                  | Bewertung \( f_i \) |
+|-----------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------|---------------------|
+| "cognitive-load-theorie   = wie wir Lernmaterialien nutzen  wie Informationen aus dem Arbeitsgedächtnis verarbeitet werden, dies ist begrenzt ... daher weniger Text, da man sich vorgelesenen Text besser merken kann (siehe Cognitive Theory of Multimedia)"                                          | 1                   |
+| "Das ICAP-Modell von Chi &amp; Wylie  ... daher nicht nur präsentieren, sondern auch interaktive Aktivitäten (Kleingruppen) ! ... Zuletzt würde ich nach dem IPAC- Modell noch eine Diskussion starten, so dass die bis dahin nur Zuhörenden interaktiv sich austauschen und ihre Gedankengänge dazu sagen können." | 1                   |
+| "Multimedia = bild + wörter meistens ... dann Integration mit Vorwissen -&gt; dann lernen ... daher beide Kanäle ansprechen ! ... multimediales lernen ist besser!"                                                                                                                                          | 1                   |
+| "Evidenzbasierte Prinzipien zur Gestaltung von multimedialen Inhalten  Powerpointfolien im Vortrag - grafische Darstellung ... Infos räumlich nah und relativ nah im zeitlichen abstand"                                                                                                                   | 1                   |
+| "Mit den jetzigen Informationen würde ich meine Präsentation mit einer PowerPoint untermalen, auf welcher überwiegend Bilder zu sehen sind, welche ich gleichzeitig mit Worten erkläre ... daher würde ich alle Lernaktivitäten miteinander vereinen, um den bestmöglichen Vortrag zu haben."                | 1                   |
+| **Gesamtbewertung**                                                                                                                                                                                                                                                                                       | 5                   |</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">

</xml_diff>